<commit_message>
更新 README / AI_HANDOFF / 卡牌清单
- README.md: 新增事件系统、装备堆叠、管理员跳过战斗等条目，更新卡牌统计
- AI_HANDOFF.md: 新增8.5节事件系统完整文档，更新装备堆叠、地图密度、交互流程等全部章节
- 卡牌清单.xlsx: 24张卡牌名称同步docx新命名
</commit_message>
<xml_diff>
--- a/卡牌清单.xlsx
+++ b/卡牌清单.xlsx
@@ -703,7 +703,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>干姜</t>
+          <t>干姜温中</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>半夏</t>
+          <t>半夏燥湿</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>苦桔梗</t>
+          <t>桔梗宣肺</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>熟地黄</t>
+          <t>熟地滋阴</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>薄荷</t>
+          <t>薄荷疏风</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>莪术</t>
+          <t>莪术破积</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>三棱</t>
+          <t>三棱破血</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>淡豆豉</t>
+          <t>豆豉宣郁</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>牛蒡子</t>
+          <t>牛蒡解毒</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>苏叶</t>
+          <t>苏叶解表</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>柴胡</t>
+          <t>柴胡疏肝</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>五味子</t>
+          <t>五味敛阴</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -4753,7 +4753,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>人参</t>
+          <t>人参补气</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>细辛</t>
+          <t>细辛通窍</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>杏仁</t>
+          <t>杏仁降气</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -5212,7 +5212,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>蒲公英</t>
+          <t>蒲公英消肿</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>天门冬</t>
+          <t>天冬养阴</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>荆芥穗</t>
+          <t>芥穗散风</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>葛根</t>
+          <t>葛根解肌</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>赤芍</t>
+          <t>赤芍凉血</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>厚朴</t>
+          <t>厚朴行气</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>生石膏</t>
+          <t>石膏清热</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>竹叶</t>
+          <t>竹叶清心</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>苍术</t>
+          <t>苍术健脾</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">

</xml_diff>

<commit_message>
doc: 同步 README / AI_HANDOFF / 卡牌清单到 v2.4
- README: 新增事件线性队列/战斗轮换/管理员密码/敌人不重复条目，地图结构重写
- AI_HANDOFF: §1定位更新线性事件, §8.5调度逻辑重写, §11密度表更新, §21新增6项变更
- 卡牌清单: 统计页刷新85/12/11/10, 新增事件队列/地图密度/管理员密码条目
</commit_message>
<xml_diff>
--- a/卡牌清单.xlsx
+++ b/卡牌清单.xlsx
@@ -7597,7 +7597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7622,17 +7622,17 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>装备</t>
+          <t>药材牌</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>11</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>药方</t>
+          <t>药方牌</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -7642,11 +7642,69 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>装备牌</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>85</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>敌方机制牌</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>事件</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1主线(3幕) + 11支线</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>事件队列</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>线性(Act1→Act2→Act3→支线)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>地图密度</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>85%事件/10%商店/5%战斗</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>管理员密码</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>260208</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update shop counts and project docs
</commit_message>
<xml_diff>
--- a/卡牌清单.xlsx
+++ b/卡牌清单.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,9 @@
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <b val="1"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
@@ -88,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,6 +102,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1423,7 +1438,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2748,7 +2763,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3832,7 +3847,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -5091,7 +5106,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -5282,7 +5297,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -5343,7 +5358,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -5794,7 +5809,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -6326,7 +6341,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -6647,7 +6662,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -6834,7 +6849,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>药材</t>
+          <t>敌方机制</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -7597,113 +7612,186 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>分类统计</t>
         </is>
       </c>
+      <c r="B1" s="6" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>分类</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>药材牌</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>85</v>
+      <c r="B3" s="8" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>药方牌</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="8" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>装备牌</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="8" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>敌方机制牌</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="9" t="n">
         <v>10</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
+    </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>事件</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>1主线(3幕) + 11支线</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>事件队列</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>线性(Act1→Act2→Act3→支线)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>地图密度</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>85%事件/10%商店/5%战斗</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>管理员密码</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>260208</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>药房合成</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>显示牌组/手牌/材料数量；每张候选牌显示同模板拥有数量xN（含x1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>三兄弟Act1二哥</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>生命上限+2，金币+50（替代满血开局回血）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>资源加载</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>主页加载进度总量只统计critical/static预加载资源，不计入未预载GIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>测试</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14：6个测试文件 / 71个测试通过；npm run build通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>更新日期</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>

</xml_diff>